<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-08 Le cartable de Raphaël
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-08.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-08.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>couloir à l'horloge, école, porte du soir</t>
+          <t>école puis maison, cartable contre le bois de la porte, horloge du couloir, poussière</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Raphaël, papa, maman, maîtresse</t>
+          <t>Raphaël, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Raphaël veut porter le cartable lourd jusqu'à l'école. L'horloge fait tic. Un chuchotement serre son ventre. Le soir, il raconte, et on remplit la gourde pour demain.</t>
+          <t>Une poussière dore près du bois de la porte. Sur le fermoir, un éclat de cartable brille. Raphaël veut parler maintenant. Il coupe papa : les mots se perdent. Le cartable penche. À l'école, un secret serre le ventre ; sa phrase se cogne à la classe. Il refuse de foncer, attend le silence, raconte. Merci vécu. Sur le fermoir, l'éclat de cartable tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le cartable s'appuie contre le bois de la porte. Le bois est froid, un peu lisse. L'horloge du couloir fait tic, tic. Une poussière dore dans le rayon du matin. Maman noue les lacets, un nœud, puis l'autre. Papa glisse une gourde dans la poche. Ça sent le cuir du cartable et le pain du petit déjeuner. L'horloge a une voix, tu l'entends ? Tic, tic. Elle est lente. Elle nous dit : c'est l'heure. En ce moment, Raphaël écoute le tic de l'horloge. Il pose la main sur le cartable. Le tissu est rêche. Il est lourd, papa. Je veux le porter jusqu'à l'école. La gourde est dedans. On le porte ensemble jusqu'à la porte. Raphaël soulève le cartable. Il avance d'un pas, puis un autre. Tu dis bonjour à la maîtresse. Et merci à la fin. Oui, maman. L'école sent les feutres. Les casiers claquent tout doux. Bonjour. On range les feutres. Bonjour, maîtresse. Raphaël écoute. Il range son feutre orange, le bouchon bien enfoncé. L'orange sent fort, comme une peau d'agrume. Merci, Raphaël. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Il écoute encore la classe, tout près de sa chaise. Il se souvient du tic de l'horloge, à la maison. Le soir, le cartable s'appuie encore contre la porte. L'horloge fait tic, tic, plus lent, plus doux. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est encore rêche. Le ventre est encore serré.</t>
+          <t>Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un éclat de cartable brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix parle bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le cartable s'appuie contre le bois de la porte. Le bois est froid, un peu lisse. L'horloge du couloir fait tic, tic. Une poussière dore dans le rayon du matin. Maman noue les lacets, un nœud, puis l'autre. Papa glisse une gourde dans la poche. Ça sent le cuir du cartable et le pain du petit déjeuner. L'horloge a une voix, tu l'entends ? Tic, tic. Elle est lente. Elle nous dit : c'est l'heure. En ce moment, Raphaël écoute le tic de l'horloge. Il pose la main sur le cartable. Le tissu est rêche. Il est lourd, papa. Je veux le porter jusqu'à l'école. La gourde est dedans. On le porte ensemble jusqu'à la porte. Raphaël soulève le cartable. Il avance d'un pas, puis un autre. Tu dis bonjour à la maîtresse. Et merci à la fin. Oui, maman. L'école sent les feutres. Les casiers claquent tout doux. Bonjour. On range les feutres. Bonjour, maîtresse. Raphaël écoute. Il range son feutre orange, le bouchon bien enfoncé. L'orange sent fort, comme une peau d'agrume. Merci, Raphaël. Plus tard, quelqu'un s'approche. Une voix parle tout bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Il écoute encore la classe, tout près de sa chaise. Il se souvient du tic de l'horloge, à la maison. Le soir, le cartable s'appuie encore contre la porte. L'horloge fait tic, tic, plus lent, plus doux. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est encore rêche. Le ventre est encore serré.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un &lt;emphasis level="moderate"&gt;éclat de cartable&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix parle bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ewen est à l'école. La maîtresse parle. Ewen aime &lt;emphasis&gt;écouter&lt;/emphasis&gt;. La maîtresse dit : on range les feutres. Ewen range son feutre. Il écoute bien. Plus tard, un camarade chuchote. Il dit : c'est un secret. Garde ça pour toi. Ewen sent un malaise. Son ventre est serré. Le soir, papa l'attend. Ewen vient raconter à la maison. Il dit : papa, j'ai eu un malaise. Un camarade a parlé d'un secret. Papa l'écoute. Papa dit : tu as bien fait. On aime écouter la maîtresse. Si tu as un malaise, tu viens raconter à papa ou maman. [pause]</t>
+          <t>Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un &lt;emphasis&gt;éclat de cartable&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix parle bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>écouter</t>
+          <t>éclat de cartable</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,55 +1321,86 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_parler_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le cartable s'appuie contre le bois de la porte.
+          <t>narrateur|Une poussière dore près du bois de la porte.
 narrateur|Le bois est froid, un peu lisse.
-narrateur|L'horloge du couloir fait tic, tic.
-narrateur|Une poussière dore dans le rayon du matin.
-narrateur|Maman noue les lacets, un nœud, puis l'autre.
+narrateur|Le cartable s'appuie contre ce bois.
+narrateur|Sur le fermoir, un éclat de cartable brille.
+enfant-m|Il est blanc, papa.
+papa|C'est le cuir, sous la lumière.
 narrateur|Papa glisse une gourde dans la poche.
-narrateur|Ça sent le cuir du cartable et le pain du petit déjeuner.
-maman|L'horloge a une voix, tu l'entends ?
-enfant-m|Tic, tic.
+maman|Tes lacets, Raphaël ?
+narrateur|Maman noue un lacet, puis l'autre.
+narrateur|Ça sent le cuir du cartable.
+narrateur|L'horloge du couloir fait tic.
+maman|Tu l'entends, Raphaël ?
+enfant-m|Tic.
 enfant-m|Elle est lente.
-papa|Elle nous dit : c'est l'heure.
-narrateur|En ce moment, Raphaël écoute le tic de l'horloge.
-narrateur|Il pose la main sur le cartable.
-narrateur|Le tissu est rêche.
-enfant-m|Il est lourd, papa.
-enfant-m|Je veux le porter jusqu'à l'école.
-papa|La gourde est dedans.
-papa|On le porte ensemble jusqu'à la porte.
-narrateur|Raphaël soulève le cartable.
-narrateur|Il avance d'un pas, puis un autre.
-maman|Tu dis bonjour à la maîtresse.
-maman|Et merci à la fin.
+papa|Elle dit l'heure.
+enfant-m|Papa, le fermoir brille, maintenant !
+narrateur|Papa parle à maman, près de la gourde.
+papa|La gourde est pleine, pour midi.
+narrateur|Les mots de Raphaël se cognent à ceux de papa.
+narrateur|Personne ne tourne la tête.
+papa|Tu disais quelque chose, Raphaël ?
+enfant-m|Le fermoir.
+enfant-m|Il brille.
+narrateur|En ce moment, Raphaël pose la main sur le cartable.
+narrateur|Le tissu est rêche, un peu lourd.
+enfant-m|Je le porte, maintenant !
+narrateur|Il soulève le cartable trop vite.
+narrateur|Le fermoir claque.
+narrateur|La gourde penche dans la poche.
+enfant-m|Oh.
+narrateur|L'éclat de cartable tremble, puis tient.
+narrateur|Le sourire de Raphaël disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-m|Ça ne veut pas, maman.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa se baisse à sa hauteur.
+papa|On le porte ensemble ?
+enfant-m|Oui, papa.
+narrateur|Ils avancent jusqu'à la porte.
+maman|Tu dis bonjour, à l'école ?
 enfant-m|Oui, maman.
+enfant-m|Au revoir, maman.
+maman|Au revoir, Raphaël.
+narrateur|Dehors, la rue brille un peu.
 narrateur|L'école sent les feutres.
-narrateur|Les casiers claquent tout doux.
-maitresse|Bonjour.
-maitresse|On range les feutres.
+narrateur|Un feutre orange attend sur la table.
+narrateur|La maîtresse parle près des chaises.
 enfant-m|Bonjour, maîtresse.
-narrateur|Raphaël écoute.
-narrateur|Il range son feutre orange, le bouchon bien enfoncé.
-narrateur|L'orange sent fort, comme une peau d'agrume.
-maitresse|Merci, Raphaël.
+narrateur|Raphaël glisse le feutre dans la boîte.
+narrateur|Le bouchon est enfoncé, bien fermé.
+narrateur|L'orange sent fort, comme une peau.
 narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle tout bas, d'un secret.
+narrateur|Une voix parle bas, d'un secret.
 narrateur|Raphaël sent un malaise.
 narrateur|Son ventre se serre.
-narrateur|Il écoute encore la classe, tout près de sa chaise.
-narrateur|Il se souvient du tic de l'horloge, à la maison.
-narrateur|Le soir, le cartable s'appuie encore contre la porte.
-narrateur|L'horloge fait tic, tic, plus lent, plus doux.
+enfant-m|Je le dis, maintenant !
+narrateur|Il ouvre la bouche trop vite.
+narrateur|Ses mots se cognent à la classe.
+narrateur|Personne ne comprend.
+narrateur|Raphaël referme la bouche.
+narrateur|Il serre les mains sur la table.
+narrateur|Il se souvient du tic, à la maison.
+narrateur|Le soir, le cartable s'appuie contre la porte.
+narrateur|L'horloge du couloir fait tic.
+narrateur|La poussière dore, plus basse.
 narrateur|La porte s'ouvre.
 papa|Te voilà.
 papa|La gourde est vide ?
 narrateur|Raphaël pose le cartable.
-narrateur|Le tissu est encore rêche.
-narrateur|Le ventre est encore serré.</t>
+narrateur|Le tissu est rêche.
+narrateur|Le ventre est serré, minuscule.
+narrateur|Il regarde papa.
+narrateur|Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1406,12 +1437,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a un malaise. Que fait-il ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Raphaël a un &lt;emphasis level="moderate"&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Ewen a un malaise. Que fait-il ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Raphaël a un &lt;emphasis&gt;malaise&lt;/emphasis&gt;. Que fait-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1474,7 +1505,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1482,10 +1513,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1500,34 +1531,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>malaise</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1536,23 +1571,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=il_raconte_quand_on_l_entend; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1585,17 +1620,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Papa. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens près de l'horloge. Raphaël parle. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. L'horloge m'a rappelé la maison. Et tu es venu nous le dire. Le ventre de Raphaël se desserre, au rythme du tic.</t>
+          <t>Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le silence arrive. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Papa. J'ai eu un malaise. Quelqu'un a parlé d'un secret. On t'écoute. Viens près de l'horloge. Raphaël parle. Papa écoute. Maman écoute. Tu as bien fait de raconter. À l'école, on écoute la maîtresse. Si tu as un malaise, tu viens le dire. L'horloge m'a rappelé la maison. Et tu es venu nous le dire. Le ventre de Raphaël se desserre, au rythme du tic.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ewen a écouté la maîtresse. Il a raconté son malaise à la maison. Papa est là. [pause]</t>
+          <t>Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1642,7 +1677,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1650,10 +1685,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1674,28 +1709,32 @@
       <c r="AG4" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>silence</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1704,10 +1743,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,25 +1759,42 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_attend_puis_on_l_entend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>enfant-m|Papa.
+          <t>narrateur|Raphaël ouvre la bouche trop vite.
+enfant-m|Papa, un secret.
+narrateur|Papa n'a pas fini sa phrase.
+papa|La gourde est vide, Raphaël.
+narrateur|Les deux voix se mélangent.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Raphaël refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Il pose les mains à plat.
+papa|Tes lacets sont un peu poussiéreux.
+narrateur|Papa pose la gourde sur le bois.
+maman|L'eau peut attendre.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Raphaël attend que le silence arrive.
+narrateur|Sur le fermoir, l'éclat de cartable brille.
+enfant-m|Il est là.
+enfant-m|Je peux te dire quelque chose ?
+maman|Oui, nous t'écoutons.
+enfant-m|Un camarade a parlé d'un secret.
 enfant-m|J'ai eu un malaise.
-enfant-m|Quelqu'un a parlé d'un secret.
-papa|On t'écoute.
-maman|Viens près de l'horloge.
-narrateur|Raphaël parle.
-narrateur|Papa écoute.
-narrateur|Maman écoute.
-papa|Tu as bien fait de raconter.
-maman|À l'école, on écoute la maîtresse.
-papa|Si tu as un malaise, tu viens le dire.
-enfant-m|L'horloge m'a rappelé la maison.
-papa|Et tu es venu nous le dire.
-narrateur|Le ventre de Raphaël se desserre, au rythme du tic.</t>
+papa|Merci, Raphaël.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu as soif ?
+enfant-m|Un peu, maman.
+narrateur|Le ventre de Raphaël se desserre.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>porte,cartable</t>
         </is>
       </c>
     </row>
@@ -1765,17 +1821,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Maman prend la gourde. L'eau chante dans le goulot. On la remplit pour demain ? Oui, maman. Raphaël tient la gourde des deux mains. Elle redevient lourde, un peu froide. Tu la glisses dans la poche ? Oui. Le cartable reprend son poids. Raphaël l'appuie contre le bois. Tic, tic. Elle dit : demain, c'est encore l'heure. On reste encore un peu dans le couloir ? Oui, papa. La poussière dore encore, plus bas.</t>
+          <t>Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la gourde trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Maman prend la gourde. L'eau chante dans le goulot. On la remplit pour demain ? Oui, maman. Raphaël tient la gourde des deux mains. Elle redevient lourde, un peu froide. Tu la glisses dans la poche ? Oui. Le cartable reprend son poids. Raphaël l'appuie contre le bois. Tic, tic. Elle dit : demain, c'est encore l'heure. On reste encore un peu dans le couloir ? Oui, papa. La poussière dore encore, plus bas.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la &lt;emphasis level="moderate"&gt;gourde&lt;/emphasis&gt; trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ewen boit un verre d'eau. Papa lui tient la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la &lt;emphasis&gt;gourde&lt;/emphasis&gt; trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1822,7 +1878,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1830,10 +1886,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1856,30 +1912,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>gourde</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1888,10 +1944,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1902,24 +1958,41 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_sur_la_gourde; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Maman prend la gourde.
-narrateur|L'eau chante dans le goulot.
-maman|On la remplit pour demain ?
-enfant-m|Oui, maman.
-narrateur|Raphaël tient la gourde des deux mains.
-narrateur|Elle redevient lourde, un peu froide.
-papa|Tu la glisses dans la poche ?
+          <t>narrateur|Raphaël veut dire le reste tout de suite.
+enfant-m|Il a dit : garde ça.
+narrateur|Il saisit la gourde trop vite.
+narrateur|L'eau penche vers le goulot.
+enfant-m|Oh.
+narrateur|Les mots se perdent dans le couloir.
+narrateur|Raphaël s'arrête.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Il refuse de foncer.
+narrateur|Il pose la gourde sur le bois.
+narrateur|Il écoute le tic, un instant.
+enfant-m|Le secret m'a serré le ventre.
+papa|Tu le poses, le cartable ?
 enfant-m|Oui.
-narrateur|Le cartable reprend son poids.
-narrateur|Raphaël l'appuie contre le bois.
-enfant-m|Tic, tic.
-maman|Elle dit : demain, c'est encore l'heure.
-papa|On reste encore un peu dans le couloir ?
+narrateur|Raphaël appuie le cartable contre la porte.
+maman|La gourde, pour demain ?
+enfant-m|Je la remplis.
+narrateur|Maman verse l'eau.
+narrateur|Ça fait un petit bruit.
+narrateur|Raphaël glisse la gourde dans la poche.
+papa|Le fermoir, tu le vois ?
 enfant-m|Oui, papa.
-narrateur|La poussière dore encore, plus bas.</t>
+narrateur|Le bois tient le cuir, sans bouger.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>gourde,eau</t>
         </is>
       </c>
     </row>
@@ -1946,17 +2019,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le cartable attend contre la porte. L'horloge fait tic, tout doux. On t'a écouté, Raphaël. La gourde est pleine, pour demain.</t>
+          <t>Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'éclat de cartable tient sur le fermoir.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le cartable attend contre la porte. L'horloge fait tic, tout doux. On t'a écouté, Raphaël. La gourde est pleine, pour demain.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'&lt;emphasis level="moderate"&gt;éclat de cartable&lt;/emphasis&gt; tient sur le fermoir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'&lt;emphasis&gt;éclat de cartable&lt;/emphasis&gt; tient sur le fermoir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2003,7 +2076,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2011,10 +2084,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2023,12 +2096,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2037,17 +2110,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cartable</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2056,11 +2133,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2069,27 +2146,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fermoir; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
           <t>narrateur|Le cartable attend contre la porte.
-narrateur|L'horloge fait tic, tout doux.
-papa|On t'a écouté, Raphaël.
-maman|La gourde est pleine, pour demain.</t>
+narrateur|L'horloge du couloir fait tic, plus loin.
+enfant-m|Il a fait tout le chemin.
+papa|Toi aussi.
+narrateur|La poussière dore, basse, près du bois.
+maman|Tu souffles ?
+enfant-m|Oui, maman.
+narrateur|Raphaël souffle.
+narrateur|Le ventre est large, à sa place.
+maman|On est bien, ici.
+papa|La gourde est pleine, pour demain.
+enfant-m|Je la verrai.
+narrateur|Le tic remplit le couloir.
+narrateur|L'éclat de cartable tient sur le fermoir.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte,horloge</t>
         </is>
       </c>
     </row>
@@ -2110,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2167,6 +2263,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-COL.ECO.001-08 Le cartable de Raphaël (polish)
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-COL.ECO.001-08.xlsx
+++ b/stories/arbres/ATOM-COL.ECO.001-08.xlsx
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un éclat de cartable brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix parle bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche.</t>
+          <t>Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un éclat de cartable brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa et de maman. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie de parler et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises, d'une voix claire. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix d'enfant parle bas, près de l'oreille, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic de l'horloge, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un &lt;emphasis level="moderate"&gt;éclat de cartable&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix parle bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un &lt;emphasis level="moderate"&gt;éclat de cartable&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa et de maman. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie de parler et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises, d'une voix claire. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix d'enfant parle bas, près de l'oreille, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic de l'horloge, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un &lt;emphasis&gt;éclat de cartable&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix parle bas, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche. [pause]</t>
+          <t>Une poussière dore près du bois de la porte. Le bois est froid, un peu lisse. Le cartable s'appuie contre ce bois. Sur le fermoir, un &lt;emphasis&gt;éclat de cartable&lt;/emphasis&gt; brille. Il est blanc, papa. C'est le cuir, sous la lumière. Papa glisse une gourde dans la poche. Tes lacets, Raphaël ? Maman noue un lacet, puis l'autre. Ça sent le cuir du cartable. L'horloge du couloir fait tic. Tu l'entends, Raphaël ? Tic. Elle est lente. Elle dit l'heure. Papa, le fermoir brille, maintenant ! Papa parle à maman, près de la gourde. La gourde est pleine, pour midi. Les mots de Raphaël se cognent à ceux de papa et de maman. Personne ne tourne la tête. Tu disais quelque chose, Raphaël ? Le fermoir. Il brille. En ce moment, Raphaël pose la main sur le cartable. Le tissu est rêche, un peu lourd. Je le porte, maintenant ! Il soulève le cartable trop vite. Le fermoir claque. La gourde penche dans la poche. Oh. L'éclat de cartable tremble, puis tient. Le sourire de Raphaël disparaît. Dans sa poitrine, l'envie de parler et l'inquiétude se bousculent. Ça ne veut pas, maman. Ses épaules tombent un peu. Papa se baisse à sa hauteur. On le porte ensemble ? Oui, papa. Ils avancent jusqu'à la porte. Tu dis bonjour, à l'école ? Oui, maman. Au revoir, maman. Au revoir, Raphaël. Dehors, la rue brille un peu. L'école sent les feutres. Un feutre orange attend sur la table. La maîtresse parle près des chaises, d'une voix claire. Bonjour, maîtresse. Raphaël glisse le feutre dans la boîte. Le bouchon est enfoncé, bien fermé. L'orange sent fort, comme une peau. Plus tard, quelqu'un s'approche. Une voix d'enfant parle bas, près de l'oreille, d'un secret. Raphaël sent un malaise. Son ventre se serre. Je le dis, maintenant ! Il ouvre la bouche trop vite. Ses mots se cognent à la classe. Personne ne comprend. Raphaël referme la bouche. Il serre les mains sur la table. Il se souvient du tic de l'horloge, à la maison. Le soir, le cartable s'appuie contre la porte. L'horloge du couloir fait tic. La poussière dore, plus basse. La porte s'ouvre. Te voilà. La gourde est vide ? Raphaël pose le cartable. Le tissu est rêche. Le ventre est serré, minuscule. Il regarde papa. Il ouvre la bouche. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1346,7 +1346,7 @@
 enfant-m|Papa, le fermoir brille, maintenant !
 narrateur|Papa parle à maman, près de la gourde.
 papa|La gourde est pleine, pour midi.
-narrateur|Les mots de Raphaël se cognent à ceux de papa.
+narrateur|Les mots de Raphaël se cognent à ceux de papa et de maman.
 narrateur|Personne ne tourne la tête.
 papa|Tu disais quelque chose, Raphaël ?
 enfant-m|Le fermoir.
@@ -1360,7 +1360,7 @@
 enfant-m|Oh.
 narrateur|L'éclat de cartable tremble, puis tient.
 narrateur|Le sourire de Raphaël disparaît.
-narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Dans sa poitrine, l'envie de parler et l'inquiétude se bousculent.
 enfant-m|Ça ne veut pas, maman.
 narrateur|Ses épaules tombent un peu.
 narrateur|Papa se baisse à sa hauteur.
@@ -1374,13 +1374,13 @@
 narrateur|Dehors, la rue brille un peu.
 narrateur|L'école sent les feutres.
 narrateur|Un feutre orange attend sur la table.
-narrateur|La maîtresse parle près des chaises.
+narrateur|La maîtresse parle près des chaises, d'une voix claire.
 enfant-m|Bonjour, maîtresse.
 narrateur|Raphaël glisse le feutre dans la boîte.
 narrateur|Le bouchon est enfoncé, bien fermé.
 narrateur|L'orange sent fort, comme une peau.
 narrateur|Plus tard, quelqu'un s'approche.
-narrateur|Une voix parle bas, d'un secret.
+narrateur|Une voix d'enfant parle bas, près de l'oreille, d'un secret.
 narrateur|Raphaël sent un malaise.
 narrateur|Son ventre se serre.
 enfant-m|Je le dis, maintenant !
@@ -1389,7 +1389,7 @@
 narrateur|Personne ne comprend.
 narrateur|Raphaël referme la bouche.
 narrateur|Il serre les mains sur la table.
-narrateur|Il se souvient du tic, à la maison.
+narrateur|Il se souvient du tic de l'horloge, à la maison.
 narrateur|Le soir, le cartable s'appuie contre la porte.
 narrateur|L'horloge du couloir fait tic.
 narrateur|La poussière dore, plus basse.
@@ -1620,17 +1620,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le silence arrive. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre.</t>
+          <t>Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le silence arrive près du cartable. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase, sans la couper. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le &lt;emphasis level="moderate"&gt;silence&lt;/emphasis&gt; arrive près du cartable. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase, sans la couper. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre. [pause]</t>
+          <t>Raphaël ouvre la bouche trop vite. Papa, un secret. Papa n'a pas fini sa phrase. La gourde est vide, Raphaël. Les deux voix se mélangent. Oh. Le sourire ne revient pas. Raphaël refuse de foncer. Il referme la bouche. Il pose les mains à plat. Tes lacets sont un peu poussiéreux. Papa pose la gourde sur le bois. L'eau peut attendre. Maman n'a pas fini non plus. Raphaël attend que le &lt;emphasis&gt;silence&lt;/emphasis&gt; arrive près du cartable. Sur le fermoir, l'éclat de cartable brille. Il est là. Je peux te dire quelque chose ? Oui, nous t'écoutons. Un camarade a parlé d'un secret. J'ai eu un malaise. Merci, Raphaël. Papa a entendu toute la phrase, sans la couper. Tu as soif ? Un peu, maman. Le ventre de Raphaël se desserre. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1778,7 +1778,7 @@
 narrateur|Papa pose la gourde sur le bois.
 maman|L'eau peut attendre.
 narrateur|Maman n'a pas fini non plus.
-narrateur|Raphaël attend que le silence arrive.
+narrateur|Raphaël attend que le silence arrive près du cartable.
 narrateur|Sur le fermoir, l'éclat de cartable brille.
 enfant-m|Il est là.
 enfant-m|Je peux te dire quelque chose ?
@@ -1786,7 +1786,7 @@
 enfant-m|Un camarade a parlé d'un secret.
 enfant-m|J'ai eu un malaise.
 papa|Merci, Raphaël.
-narrateur|Papa a entendu toute la phrase.
+narrateur|Papa a entendu toute la phrase, sans la couper.
 maman|Tu as soif ?
 enfant-m|Un peu, maman.
 narrateur|Le ventre de Raphaël se desserre.</t>
@@ -1821,17 +1821,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la gourde trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger.</t>
+          <t>Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la gourde trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir, sous le tic. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la &lt;emphasis level="moderate"&gt;gourde&lt;/emphasis&gt; trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la &lt;emphasis level="moderate"&gt;gourde&lt;/emphasis&gt; trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir, sous le tic. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la &lt;emphasis&gt;gourde&lt;/emphasis&gt; trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger. [pause]</t>
+          <t>Raphaël veut dire le reste tout de suite. Il a dit : garde ça. Il saisit la &lt;emphasis&gt;gourde&lt;/emphasis&gt; trop vite. L'eau penche vers le goulot. Oh. Les mots se perdent dans le couloir, sous le tic. Raphaël s'arrête. Ses mains se ferment, puis s'ouvrent. Il refuse de foncer. Il pose la gourde sur le bois. Il écoute le tic, un instant. Le secret m'a serré le ventre. Tu le poses, le cartable ? Oui. Raphaël appuie le cartable contre la porte. La gourde, pour demain ? Je la remplis. Maman verse l'eau. Ça fait un petit bruit. Raphaël glisse la gourde dans la poche. Le fermoir, tu le vois ? Oui, papa. Le bois tient le cuir, sans bouger. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1970,7 +1970,7 @@
 narrateur|Il saisit la gourde trop vite.
 narrateur|L'eau penche vers le goulot.
 enfant-m|Oh.
-narrateur|Les mots se perdent dans le couloir.
+narrateur|Les mots se perdent dans le couloir, sous le tic.
 narrateur|Raphaël s'arrête.
 narrateur|Ses mains se ferment, puis s'ouvrent.
 narrateur|Il refuse de foncer.
@@ -2019,17 +2019,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'éclat de cartable tient sur le fermoir.</t>
+          <t>Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois de la porte. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'éclat de cartable tient sur le fermoir.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'&lt;emphasis level="moderate"&gt;éclat de cartable&lt;/emphasis&gt; tient sur le fermoir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois de la porte. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'&lt;emphasis level="moderate"&gt;éclat de cartable&lt;/emphasis&gt; tient sur le fermoir.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'&lt;emphasis&gt;éclat de cartable&lt;/emphasis&gt; tient sur le fermoir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le cartable attend contre la porte. L'horloge du couloir fait tic, plus loin. Il a fait tout le chemin. Toi aussi. La poussière dore, basse, près du bois de la porte. Tu souffles ? Oui, maman. Raphaël souffle. Le ventre est large, à sa place. On est bien, ici. La gourde est pleine, pour demain. Je la verrai. Le tic remplit le couloir. L'&lt;emphasis&gt;éclat de cartable&lt;/emphasis&gt; tient sur le fermoir.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
 narrateur|L'horloge du couloir fait tic, plus loin.
 enfant-m|Il a fait tout le chemin.
 papa|Toi aussi.
-narrateur|La poussière dore, basse, près du bois.
+narrateur|La poussière dore, basse, près du bois de la porte.
 maman|Tu souffles ?
 enfant-m|Oui, maman.
 narrateur|Raphaël souffle.
@@ -2206,7 +2206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2270,6 +2270,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>